<commit_message>
Added exponential generator, graphs, tables saved as png
</commit_message>
<xml_diff>
--- a/test_1cal.xlsx
+++ b/test_1cal.xlsx
@@ -125,11 +125,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:B4" headerRowCount="1">
-  <autoFilter ref="A1:B4"/>
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabella1" displayName="Tabella1" ref="A1:D5" headerRowCount="1">
+  <autoFilter ref="A1:D5"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="Oscilloscopio"/>
     <tableColumn id="2" name="Multimetro"/>
+    <tableColumn id="3" name="Errore oscilloscopio"/>
+    <tableColumn id="4" name="Errore multimetro"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -424,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,6 +440,16 @@
           <t>Multimetro</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Errore oscilloscopio</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Errore multimetro</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -446,6 +458,12 @@
       <c r="B2" t="n">
         <v>8</v>
       </c>
+      <c r="C2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -454,6 +472,12 @@
       <c r="B3" t="n">
         <v>20</v>
       </c>
+      <c r="C3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -461,6 +485,26 @@
       </c>
       <c r="B4" t="n">
         <v>26</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>